<commit_message>
Add the Taiwan Biobank external validation Scores the 92,734-participant Taiwan Biobank cohort with the top-20 CatBoost: 19,596 predicted insulin resistant (21.1%), of whom 246 fall in the 1,199-member methylation subset. This cohort measures no fasting insulin, so it carries no observed label and no accuracy can be computed on it; what is reported instead is a predicted prevalence and two distributional comparisons against the labelled cohorts. Cohen's d on TG/HDL-C is -0.13. - src/models/evaluate.py: predict_labels(), cohens_d() - src/viz/figures.py: plot_tg_hdl_boxplots(), plot_quantile_comparison() - notebooks/07_twb_validation.ipynb plot_tg_hdl_boxplots takes a mapping of panel title to cohort, so a panel cannot show a different cohort from the one its title names.
</commit_message>
<xml_diff>
--- a/data/output/stats.xlsx
+++ b/data/output/stats.xlsx
@@ -10,6 +10,7 @@
     <sheet name="NHANES" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="KNHANES" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="COMBINE" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="TWB(predict)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -493,10 +494,6 @@
           <t>5,183</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -519,10 +516,6 @@
           <t>2,645(51.0%)</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -545,10 +538,6 @@
           <t>2,538(49.0%)</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1341,10 +1330,6 @@
           <t>4,226</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1367,10 +1352,6 @@
           <t>2,107(49.9%)</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1393,10 +1374,6 @@
           <t>2,119(50.1%)</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2189,6 +2166,842 @@
           <t>9,409</t>
         </is>
       </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>12,320(46.0%)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7,568(43.5%)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>4,752(50.5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>14,478(54.0%)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>9,821(56.5%)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>4,657(49.5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>48.8±17.8</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>48.6±17.6</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>49.4±18.0</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BMI</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>25.7±5.3</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>23.9±3.8</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>29.2±5.9</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BODY_WAISTLINE</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>89.1±14.3</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>84.1±11.2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>98.5±14.5</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BUN</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>13.9±5.0</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>14.0±4.9</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>13.9±5.2</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.14433164293085082</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CREATININE</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0.8±0.3</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0.8±0.3</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0.8±0.3</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FASTING_GLUCOSE</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>98.6±16.9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>94.2±10.2</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>106.7±22.8</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>FASTING_INSULIN</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10.5±9.8</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>6.2±2.3</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>18.5±13.0</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>HBA1C</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>5.6±0.6</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>5.5±0.4</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>5.7±0.8</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>HDL_C</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>53.4±14.2</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>56.1±14.3</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>48.4±12.5</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HOMA-IR</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2.7±3.1</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1.5±0.5</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>4.9±4.4</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LDL_C</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>116.8±34.6</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>116.4±33.7</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>117.5±36.2</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0.01203760807670484</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MAP</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>88.4±11.5</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>87.4±11.2</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>90.4±11.7</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SGOT</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>25.1±17.1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>24.1±16.7</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>27.1±17.6</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SGPT</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>24.2±20.9</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>20.9±17.2</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>30.3±25.2</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TG</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>125.4±79.9</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>109.0±68.0</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>155.8±90.5</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>T_CHO</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>195.3±38.8</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>194.3±38.0</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>197.0±40.3</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>URIC_ACID</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>5.3±1.4</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>5.0±1.3</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>5.7±1.5</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>&lt; 0.01</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>column</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>IR-</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>IR+</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ks_p_value-</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ks_p_value+</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>t_test_p_value</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>u_test_p_value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>92,734</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>73,138</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>19,596</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
@@ -2202,17 +3015,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>12,320(46.0%)</t>
+          <t>34,859(37.6%)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>7,568(43.5%)</t>
+          <t>24,393(33.4%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>4,752(50.5%)</t>
+          <t>10,466(53.4%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -2228,17 +3041,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>14,478(54.0%)</t>
+          <t>57,875(62.4%)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>9,821(56.5%)</t>
+          <t>48,745(66.6%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4,657(49.5%)</t>
+          <t>9,130(46.6%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
@@ -2254,17 +3067,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>48.8±17.8</t>
+          <t>46.4±13.2</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>48.6±17.6</t>
+          <t>46.2±13.1</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>49.4±18.0</t>
+          <t>47.0±13.7</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -2296,17 +3109,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>25.7±5.3</t>
+          <t>23.9±3.9</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>23.9±3.8</t>
+          <t>22.7±2.9</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>29.2±5.9</t>
+          <t>28.5±3.8</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -2338,17 +3151,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>89.1±14.3</t>
+          <t>82.1±10.8</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>84.1±11.2</t>
+          <t>79.0±8.5</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>98.5±14.5</t>
+          <t>93.8±10.6</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -2380,17 +3193,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.9±5.0</t>
+          <t>12.8±3.7</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14.0±4.9</t>
+          <t>12.7±3.6</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>13.9±5.2</t>
+          <t>13.2±3.8</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -2405,7 +3218,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0.14433164293085082</t>
+          <t>&lt; 0.01</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -2422,12 +3235,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0.8±0.3</t>
+          <t>0.7±0.3</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.8±0.3</t>
+          <t>0.7±0.3</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2464,17 +3277,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>98.6±16.9</t>
+          <t>93.0±13.1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>94.2±10.2</t>
+          <t>90.2±6.8</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>106.7±22.8</t>
+          <t>103.4±22.3</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -2501,22 +3314,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FASTING_INSULIN</t>
+          <t>HBA1C</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10.5±9.8</t>
+          <t>5.6±0.5</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>6.2±2.3</t>
+          <t>5.5±0.3</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>18.5±13.0</t>
+          <t>6.0±0.8</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -2543,22 +3356,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>HBA1C</t>
+          <t>HDL_C</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>5.6±0.6</t>
+          <t>56.1±13.8</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>5.5±0.4</t>
+          <t>58.7±13.5</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>5.7±0.8</t>
+          <t>46.2±10.1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -2585,22 +3398,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>HDL_C</t>
+          <t>LDL_C</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>53.4±14.2</t>
+          <t>119.9±31.9</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>56.1±14.3</t>
+          <t>118.0±31.3</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>48.4±12.5</t>
+          <t>127.1±33.2</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -2627,22 +3440,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>HOMA-IR</t>
+          <t>MAP</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2.7±3.1</t>
+          <t>88.2±12.6</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.5±0.5</t>
+          <t>86.2±11.9</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>4.9±4.4</t>
+          <t>95.6±12.1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -2669,22 +3482,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>LDL_C</t>
+          <t>SGOT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>116.8±34.6</t>
+          <t>22.8±12.5</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>116.4±33.7</t>
+          <t>21.8±11.7</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>117.5±36.2</t>
+          <t>26.9±14.6</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -2699,7 +3512,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>0.01203760807670484</t>
+          <t>&lt; 0.01</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2711,22 +3524,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MAP</t>
+          <t>SGPT</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>88.4±11.5</t>
+          <t>23.3±20.8</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>87.4±11.2</t>
+          <t>19.1±15.4</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>90.4±11.7</t>
+          <t>38.6±29.5</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -2753,22 +3566,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SGOT</t>
+          <t>TG</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>25.1±17.1</t>
+          <t>108.2±84.3</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>24.1±16.7</t>
+          <t>91.2±56.5</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>27.1±17.6</t>
+          <t>171.6±128.9</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -2795,22 +3608,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SGPT</t>
+          <t>T_CHO</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>24.2±20.9</t>
+          <t>195.5±37.4</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>20.9±17.2</t>
+          <t>194.2±37.4</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>30.3±25.2</t>
+          <t>200.2±37.1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -2837,22 +3650,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TG</t>
+          <t>URIC_ACID</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>125.4±79.9</t>
+          <t>5.4±1.4</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>109.0±68.0</t>
+          <t>5.2±1.3</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>155.8±90.5</t>
+          <t>6.3±1.5</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2871,90 +3684,6 @@
         </is>
       </c>
       <c r="H19" t="inlineStr">
-        <is>
-          <t>&lt; 0.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>T_CHO</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>195.3±38.8</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>194.3±38.0</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>197.0±40.3</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>&lt; 0.01</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>&lt; 0.01</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>&lt; 0.01</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>&lt; 0.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>URIC_ACID</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>5.3±1.4</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>5.0±1.3</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>5.7±1.5</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>&lt; 0.01</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>&lt; 0.01</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>&lt; 0.01</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
         <is>
           <t>&lt; 0.01</t>
         </is>

</xml_diff>